<commit_message>
Email nepovinný + přihlášení přes email nebo ERP id
- User.email nullable (migrace). Stačí email NEBO erpUserId.
- Login: pole "Email nebo ERP ID", hledá uživatele dle email i erpUserId.
- createUser: email volitelný (vyžaduje email nebo ERP id + heslo).
- Zobrazení jména: fallback name -> email -> erpUserId.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EX8100641\Documents\Schvalmax\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wendulka\Documents\Webhry\schaleem\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75842973-1F33-47D9-9792-2D4461EB0AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25125" windowHeight="12300"/>
+    <workbookView xWindow="11865" yWindow="-14100" windowWidth="16200" windowHeight="11835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="2" r:id="rId1"/>
@@ -21,9 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
-    <t>UserId</t>
-  </si>
-  <si>
     <t>NejedlaP</t>
   </si>
   <si>
@@ -172,12 +170,15 @@
   </si>
   <si>
     <t>Heslo</t>
+  </si>
+  <si>
+    <t>ERP userId</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -491,7 +492,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C499"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -501,21 +502,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C2">
         <v>14045</v>
@@ -523,10 +524,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3">
         <v>24072</v>
@@ -534,10 +535,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C4">
         <v>37823</v>
@@ -545,10 +546,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>56046</v>
@@ -556,10 +557,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6">
         <v>79201</v>
@@ -567,10 +568,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7">
         <v>10801</v>
@@ -578,10 +579,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C8">
         <v>1430</v>
@@ -589,10 +590,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9">
         <v>1848</v>
@@ -600,10 +601,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C10">
         <v>2340</v>
@@ -611,10 +612,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C11">
         <v>2912</v>
@@ -622,10 +623,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12">
         <v>3570</v>
@@ -633,10 +634,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C13">
         <v>4320</v>
@@ -644,10 +645,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C14">
         <v>5168</v>
@@ -655,10 +656,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15">
         <v>6120</v>
@@ -666,10 +667,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C16">
         <v>7182</v>
@@ -677,10 +678,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17">
         <v>8360</v>
@@ -688,10 +689,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C18">
         <v>9660</v>
@@ -699,10 +700,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C19">
         <v>11088</v>
@@ -710,10 +711,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C20">
         <v>12650</v>
@@ -721,10 +722,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21">
         <v>14352</v>
@@ -732,10 +733,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C22">
         <v>16200</v>
@@ -743,10 +744,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C23">
         <v>18200</v>
@@ -754,10 +755,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24">
         <v>20358</v>
@@ -765,10 +766,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C25">
         <v>22680</v>

</xml_diff>